<commit_message>
Set Logistic and Order booking
</commit_message>
<xml_diff>
--- a/Document/New REQUIREMENT.xlsx
+++ b/Document/New REQUIREMENT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bilal\ERPRepo\Document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F91F60E-9D14-40AF-94EE-72713D7C31DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0C7E48-2DBA-48CB-B427-41E30F895AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{214A8478-E50A-4AE8-A0BB-51E392BA635B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{214A8478-E50A-4AE8-A0BB-51E392BA635B}"/>
   </bookViews>
   <sheets>
     <sheet name="Ready For Dispatched" sheetId="6" r:id="rId1"/>
@@ -724,8 +724,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{EC4A64F1-B668-4921-B303-148E9D1967A3}" name="Table7" displayName="Table7" ref="A5:J6" totalsRowShown="0">
-  <autoFilter ref="A5:J6" xr:uid="{763B0444-623B-4778-8C6E-12C42E780733}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{EC4A64F1-B668-4921-B303-148E9D1967A3}" name="Table7" displayName="Table7" ref="A6:J7" totalsRowShown="0">
+  <autoFilter ref="A6:J7" xr:uid="{763B0444-623B-4778-8C6E-12C42E780733}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{FAAB77C8-1C42-42FA-A041-C5B0F5A75C29}" name="Booking No#"/>
     <tableColumn id="2" xr3:uid="{D29BDB19-F8C2-4DF7-89ED-27900C0084D9}" name="Container No#"/>
@@ -1204,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D25DF428-5068-4BA7-8310-10B2A5137995}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="31.88671875" bestFit="1" customWidth="1"/>
@@ -1224,67 +1224,67 @@
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" t="s">
-        <v>60</v>
-      </c>
-      <c r="I5" t="s">
-        <v>61</v>
-      </c>
-      <c r="J5" t="s">
-        <v>31</v>
-      </c>
-    </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="D6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" t="s">
+        <v>59</v>
+      </c>
+      <c r="H6" t="s">
+        <v>60</v>
+      </c>
+      <c r="I6" t="s">
+        <v>61</v>
+      </c>
+      <c r="J6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s">
         <v>56</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E7" t="s">
         <v>56</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F7" t="s">
         <v>56</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G7" t="s">
         <v>56</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H7" t="s">
         <v>56</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I7" t="s">
         <v>56</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J7" t="s">
         <v>90</v>
       </c>
     </row>

</xml_diff>